<commit_message>
Update with Marques2016 direct evidence
</commit_message>
<xml_diff>
--- a/external-data/Claude2026/olig_marker_genes_lit_comparison/oligodendrocyte_marker_genes_lit_comparison.xlsx
+++ b/external-data/Claude2026/olig_marker_genes_lit_comparison/oligodendrocyte_marker_genes_lit_comparison.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Oligo Marker Genes'!$A$1:$V$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Oligo Marker Genes'!$A$1:$V$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'References'!$A$1:$F$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -299,7 +299,7 @@
 High = human-confirmed AND cited in &gt;=3 papers, OR partial-human AND cited in &gt;=5 papers.
 Medium = solid support on only one axis (e.g., a single human dataset, or broad mouse-only citation across &gt;=3 papers).
 Low = single-source and/or mouse-only support, or a significant unresolved caveat (e.g. CD44's figure-only, direction-unconfirmed claim was manually kept Low despite a single human-dataset citation).
-CAVEAT: this score reflects citation support captured WITHIN THIS TABLE's specific paper columns, not the full external literature. Some markers with strong real-world consensus (e.g. SOX10) may score lower here purely because this table's per-paper cell curation for that gene is sparse (only 2 of 15 paper columns populated) -- cross-check against the broader literature before treating a Low/Medium score as a definitive negative.</t>
+CAVEAT: this score reflects citation support captured WITHIN THIS TABLE's specific paper columns, not the full external literature. SOX10 is a useful cautionary example of how far this in-table score can lag real-world consensus: it sat at Low for most of this table's history (only 2 of 15 paper columns populated) despite being one of the most universally used human oligodendrocyte-lineage markers in the field; adding a third mouse-only citation (Marques et al. 2016) has since raised it to Medium via the 'broad mouse-only citation' rule, but it still lacks a confirmed-human citation within this table. ITPR2 remains a live example of the same limitation: extensively functionally characterized in Marques et al. (2016) yet still Low here, cited in only 2 of 15 paper columns. Cross-check against the broader literature before treating a Low/Medium score as a definitive negative.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -309,7 +309,7 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Marques S et al. (2016). Oligodendrocyte heterogeneity in the mouse juvenile and adult CNS. Science 352:1326-1329. [Not reviewed directly this session; via Valihrach et al. 2022 Table 2 - verify before citing]</t>
+        <t>Marques S et al. (2016). Oligodendrocyte heterogeneity in the mouse juvenile and adult CNS. Science 352:1326-1329. [Reviewed directly]</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V56"/>
+  <dimension ref="A1:V65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -842,7 +842,7 @@
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
-          <t>Canonical, cross-species OPC marker. Absent from the disease-focused papers' tables only because those studies report disease-associated clusters, not baseline lineage stages.</t>
+          <t>Canonical, cross-species OPC marker. Absent from the disease-focused papers' tables only because those studies report disease-associated clusters, not baseline lineage stages. Marques et al. (2016) also caution that a second, non-oligodendrocyte Pdgfra+ population -- vascular/leptomeningeal cells (VLMCs) -- exists alongside true OPCs; VLMCs have low Cspg4 and instead express Lum, Vtn, Tbx18, and Col1a2, so PDGFRA positivity alone (without CSPG4) risks VLMC contamination in bulk/FACS-based OPC isolation. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a sharp, isolated OPC peak, cross-validating the OPC attribution above and the general reliability of this heatmap for stage assignment.</t>
         </is>
       </c>
       <c r="H2" s="12" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="I2" s="12" t="inlineStr">
         <is>
-          <t>OPC</t>
+          <t>OPC (co-expressed with Cspg4; a second, low-Cspg4 Pdgfra+ population = non-oligo VLMCs, see Notes)</t>
         </is>
       </c>
       <c r="J2" s="12" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Classic proteoglycan antigen also known as NG2 (mouse gene Cspg4 = the "NG2" antigen); largely superseded by PDGFRA/BCAN/SOX6 in later transcriptomic marker panels. Mironova et al. (2026) show Cspg4/NG2 mRNA is among the most enriched OPC transcripts relative to astrocytes, microglia, and neurons, and that this expression pattern is conserved across mouse, marmoset, and human — reframing this ‘classic’ protein antigen as part of a broader, cross-species CSPG expression module (with VCAN, PTPRZ1, BCAN, ACAN) rather than a standalone marker.</t>
+          <t>Classic proteoglycan antigen also known as NG2 (mouse gene Cspg4 = the "NG2" antigen); largely superseded by PDGFRA/BCAN/SOX6 in later transcriptomic marker panels. Mironova et al. (2026) show Cspg4/NG2 mRNA is among the most enriched OPC transcripts relative to astrocytes, microglia, and neurons, and that this expression pattern is conserved across mouse, marmoset, and human — reframing this ‘classic’ protein antigen as part of a broader, cross-species CSPG expression module (with VCAN, PTPRZ1, BCAN, ACAN) rather than a standalone marker. Marques et al. (2016) note VLMCs (a distinct, non-oligodendrocyte Pdgfra+ population) express low Cspg4, reinforcing Cspg4/NG2 co-positivity as the more specific way (vs. Pdgfra alone) to confirm true OPC identity in FACS/IHC-based isolations. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a sharp, isolated OPC peak, cross-validating the OPC attribution above.</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Core member of the conserved OPC-enriched CSPG module (with CSPG4, PTPRZ1, BCAN, ACAN); single-source addition here (Mironova2026).</t>
+          <t>Core member of the conserved OPC-enriched CSPG module (with CSPG4, PTPRZ1, BCAN, ACAN); now independently listed as an OPC marker gene in a second mouse dataset (Marques et al. 2016), in addition to Mironova2026.</t>
         </is>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>Human gene symbol for the CSPG Vcan (versican). Reported by Mironova et al. (2026) as one of the most highly expressed OPC transcripts, enriched relative to astrocytes, microglia, and neurons, with the expression pattern conserved across mouse, marmoset, and human. Not separately discussed in the other papers surveyed in this table.</t>
+          <t>Human gene symbol for the CSPG Vcan (versican). Reported by Mironova et al. (2026) as one of the most highly expressed OPC transcripts, enriched relative to astrocytes, microglia, and neurons, with the expression pattern conserved across mouse, marmoset, and human. Not separately discussed in the other papers surveyed in this table. Marques et al. (2016) also list Vcan among the marker genes distinguishing OPCs (Fig. 2B), independently supporting its inclusion in this OPC-enriched CSPG module from a second, earlier mouse dataset. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms Vcan is genuinely OPC/COP-enriched, but shows a near-equal peak across both stages rather than a clean OPC-only signal -- refining the Fig. 2B-based 'OPC' attribution above to 'OPC/COP'.</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>OPC / COP (near-equal peak across both stages -- quantitative pixel analysis of Fig. S1B's single-cell heatmap; OPC and COP scores are nearly identical, both well above all later stages)</t>
         </is>
       </c>
       <c r="J4" s="12" t="inlineStr">
@@ -1168,17 +1168,17 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Long-established OPC transcript, now formally placed within a conserved cross-species CSPG expression module (Mironova2026) and independently listed as a canonical scRNA-seq OPC marker (Emery &amp; Wood 2024).</t>
+          <t>Long-established OPC transcript, independently listed as an OPC marker gene in three mouse-based sources (Marques et al. 2016; Mironova et al. 2026's cross-species CSPG module; Emery &amp; Wood 2024's canonical scRNA-seq OPC panel). This mouse-only breadth now crosses this table's &gt;=3-paper Medium threshold, though a confirmed-human citation is still absent within this table.</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Reported by Mironova et al. (2026) as one of the core OPC-enriched CSPGs, conserved across mouse, marmoset, and human. Ptprz1 is also independently listed by Emery &amp; Wood (2024) as a canonical scRNA-seq OPC transcript (alongside Pdgfra and Pcdh15, both now also in this table), so this gene has long-standing, cross-methodology support as an OPC identity gene, now directly attributable to both sources rather than only Mironova2026.</t>
+          <t>Reported by Mironova et al. (2026) as one of the core OPC-enriched CSPGs, conserved across mouse, marmoset, and human. Ptprz1 is also independently listed by Emery &amp; Wood (2024) as a canonical scRNA-seq OPC transcript (alongside Pdgfra and Pcdh15, both now also in this table), so this gene has long-standing, cross-methodology support as an OPC identity gene, now directly attributable to both sources rather than only Mironova2026. Marques et al. (2016) independently list Ptprz1 among the OPC marker genes in their original mouse scRNA-seq dataset (Fig. 2B) -- the earliest of the three mouse sources now supporting this gene in this table. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a clean OPC peak (COP a distant second), cross-validating the OPC attribution above.</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>OPC</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
@@ -1285,12 +1285,12 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Canonical OPC marker transcript with an additional, distinct functional role in OPC self-spacing/homeostasis; single-source addition here (Emery &amp; Wood 2024).</t>
+          <t>Canonical OPC marker transcript with an additional, distinct functional role in OPC self-spacing/homeostasis; now supported by two mouse sources (Marques et al. 2016's original scRNA-seq panel; Emery &amp; Wood 2024, which itself cites Marques et al. 2016 for this marker).</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>Beyond its role as an OPC marker transcript, Emery &amp; Wood (2024) note that PCDH15 mediates homeostatic self-repulsion between OPCs — recently divided daughter cells repel one another via protocadherin-15, which helps maintain the OPCs' even, tiled distribution across the CNS (citing Huang et al. 2020; Zhen et al. 2022). Not discussed in the other papers surveyed in this table.</t>
+          <t>Beyond its role as an OPC marker transcript, Emery &amp; Wood (2024) note that PCDH15 mediates homeostatic self-repulsion between OPCs — recently divided daughter cells repel one another via protocadherin-15, which helps maintain the OPCs' even, tiled distribution across the CNS (citing Huang et al. 2020; Zhen et al. 2022). Not discussed in the other papers surveyed in this table. Marques et al. (2016) list Pcdh15 directly among their own OPC marker genes (Fig. 2B) -- confirming, from the primary source itself, the citation that Emery &amp; Wood (2024) had already attributed to this paper.</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>OPC</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
@@ -1728,17 +1728,17 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Human OPC marker with immunohistochemical validation (Jäkel et al.); mechanistically a SoxD differentiation-inhibitory TF that pairs with SOX5 (Emery &amp; Wood 2024).</t>
+          <t>Now High-confidence by this table's own rule: human protein-level validation (Jäkel et al., IHC-confirmed OPC marker co-expressed with OLIG2) combined with breadth across 3 papers (Jakel2019, Emery2024, Marques2016). Note a genuine cross-species/cross-method staging nuance: Jäkel's human IHC places SOX6 at the OPC stage, whereas Marques et al. (2016)'s mouse mRNA data places Sox6 at the COP stage (grouped with Bmp4/Gpr17 as genes that keep cells undifferentiated just after the OPC-&gt;COP transition).</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Validated at the protein level as co-expressed with OLIG2 in NOGO(RTN4)-negative OPCs; significantly reduced in MS lesions and NAWM vs. control tissue. Emery &amp; Wood (2024) place SOX6 within the SoxD family (obligate partner SOX5) that antagonizes oligodendrocyte differentiation — proposed mechanisms include direct competition with SOX10 at myelin-gene regulatory elements and, in a later study cited therein, promotion of Pdgfra expression (the OPC mitogen receptor) — so elevated SOX6 in OPCs is mechanistically tied to keeping cells undifferentiated, not just a passive identity marker.</t>
+          <t>Validated at the protein level as co-expressed with OLIG2 in NOGO(RTN4)-negative OPCs; significantly reduced in MS lesions and NAWM vs. control tissue. Emery &amp; Wood (2024) place SOX6 within the SoxD family (obligate partner SOX5) that antagonizes oligodendrocyte differentiation — proposed mechanisms include direct competition with SOX10 at myelin-gene regulatory elements and, in a later study cited therein, promotion of Pdgfra expression (the OPC mitogen receptor) — so elevated SOX6 in OPCs is mechanistically tied to keeping cells undifferentiated, not just a passive identity marker. Marques et al. (2016) place Sox6 mRNA specifically at the COP stage -- among genes that 'keep oligodendrocytes undifferentiated' alongside Bmp4 and Gpr17 -- rather than at the OPC stage. This is a real discrepancy with Jäkel et al. (2019)'s human IHC data (SOX6 co-expressed with OLIG2 in OPCs, reduced in MS lesions): it may reflect a genuine cross-species difference, a difference between mRNA vs. protein timing, or simply that COP and late-OPC states are difficult to cleanly separate. This table keeps the OPC categorization (from the higher-confidence human IHC source) but flags the mouse-mRNA COP-stage placement here for anyone comparing across species/methods. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a clean COP peak, cross-validating the mouse mRNA COP-stage placement described above (as distinct from Jäkel et al.'s human protein-level OPC placement).</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Committed Precursor (mRNA marker; 'keeps oligodendrocytes undifferentiated', grouped with Bmp4 and Gpr17)</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Marks the earliest post-mitotic differentiation step in mouse; no disease-focused paper here carries it forward as a marker. Emery &amp; Wood (2024) discuss BMP4 primarily as a secreted ligand (with BMP2) that inhibits OPC differentiation via BMP receptors and SMAD-mediated induction of ID2/ID4 — a different framing from Marques' use of Bmp4 mRNA as a stage marker, but not necessarily contradictory: up-regulation at the COP transition could reflect autocrine/paracrine anti-differentiation signaling right as cells commit.</t>
+          <t>Marks the earliest post-mitotic differentiation step in mouse; no disease-focused paper here carries it forward as a marker. Emery &amp; Wood (2024) discuss BMP4 primarily as a secreted ligand (with BMP2) that inhibits OPC differentiation via BMP receptors and SMAD-mediated induction of ID2/ID4 — a different framing from Marques' use of Bmp4 mRNA as a stage marker, but not necessarily contradictory: up-regulation at the COP transition could reflect autocrine/paracrine anti-differentiation signaling right as cells commit. Directly confirmed in Marques et al. (2016)'s own Fig. 2B COP marker panel (with Sox6, Gpr17, Neu4, Nkx2-2). Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a clean COP peak, cross-validating the COP attribution above.</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -2405,12 +2405,12 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>COP-stage marker gene and differentiation-promoting transcription factor that normally antagonizes OLIG2; single-source addition here (Emery &amp; Wood 2024).</t>
+          <t>COP-stage marker gene and differentiation-promoting transcription factor that normally antagonizes OLIG2; independently listed as a COP-stage marker gene in Marques et al. (2016)'s original mouse dataset, which also notes nonproliferative Nkx2.2+ precursors (profile consistent with these COP/early-differentiating cells) in human MS lesions (citing Kuhlmann et al. 2008).</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>NKX2-2 has a dual identity in Emery &amp; Wood (2024): mechanistically, it is a transcription factor that normally antagonizes OLIG2 (the two cross-repress each other), with NFATC2/SOX10 signaling needed to overcome this and induce NKX2-2 during differentiation; separately, Nkx2-2 mRNA is also listed as a scRNA-seq marker of the COP (committed OPC precursor) stage, alongside Gpr17 and Bmp4 (both already in this table). Not discussed in the other papers surveyed here.</t>
+          <t>NKX2-2 has a dual identity in Emery &amp; Wood (2024): mechanistically, it is a transcription factor that normally antagonizes OLIG2 (the two cross-repress each other), with NFATC2/SOX10 signaling needed to overcome this and induce NKX2-2 during differentiation; separately, Nkx2-2 mRNA is also listed as a scRNA-seq marker of the COP (committed OPC precursor) stage, alongside Gpr17 and Bmp4 (both already in this table). Not discussed in the other papers surveyed here. Marques et al. (2016) independently list Nkx2-2 among their COP-stage marker genes (Fig. 2B, with Sox6/Gpr17/Bmp4/Neu4) and separately note, in their Discussion, that nonproliferative Nkx2.2+ precursors with a profile consistent with their ITPR2+/newly-differentiating cells have been observed in multiple sclerosis lesions (citing Kuhlmann et al. 2008) -- an early hint at disease relevance for this differentiation-stage transcription factor, well before the disease-associated-oligodendrocyte literature captured elsewhere in this table.</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Committed Precursor (Fig. 2B marker, grouped with Sox6/Gpr17/Bmp4/Neu4); nonproliferative Nkx2.2+ precursors also observed in MS lesions</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>Well-characterized negative regulator/'timer' of oligodendrocyte maturation (Chen et al. 2009, cited in Hughes &amp; Stockton); genetic deletion accelerates maturation. Emery &amp; Wood (2024) independently corroborate this exact mechanism, citing the same primary source (Chen et al. 2009) already anchoring the Hughes2021 column in this table.</t>
+          <t>Well-characterized negative regulator/'timer' of oligodendrocyte maturation (Chen et al. 2009, cited in Hughes &amp; Stockton); genetic deletion accelerates maturation. Emery &amp; Wood (2024) independently corroborate this exact mechanism, citing the same primary source (Chen et al. 2009) already anchoring the Hughes2021 column in this table. Directly confirmed in Marques et al. (2016)'s own Fig. 2B COP marker panel (with Sox6, Neu4, Bmp4, Nkx2-2). Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a COP peak (with NFOL1/NFOL2 also elevated, consistent with its role as a differentiation 'timer' that declines through these stages), cross-validating the COP attribution above.</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>Committed Precursor</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Transiently expressed, mechanistically biphasic (first anti-, then pro-differentiation) transcription factor; also used as an NFOL-stage scRNA-seq marker gene — single-source addition here (Emery &amp; Wood 2024).</t>
+          <t>Transiently expressed, mechanistically biphasic (first anti-, then pro-differentiation) transcription factor; used as an NFOL-stage scRNA-seq marker gene in both its original primary source (Marques et al. 2016, now directly confirmed and added to this table) and a secondary review that cites it (Emery &amp; Wood 2024).</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>TCF7L2 is highlighted by Emery &amp; Wood (2024) as a marker transiently expressed as OPCs commit to differentiating, with a genuinely biphasic mechanism: early on it partners with β-catenin to inhibit differentiation (Wnt-pathway-like action), then later switches partners (HDACs, KAISO) to instead promote differentiation together with SOX10. It is separately listed as a canonical NFOL-stage marker gene in scRNA-seq marker panels (Marques et al. 2016, cited within Emery &amp; Wood 2024) — so the same transcript spans a mechanistic role at the commitment step and a marker role slightly later, at the newly-formed-oligodendrocyte stage. Not discussed in the other papers surveyed in this table.</t>
+          <t>TCF7L2 is highlighted by Emery &amp; Wood (2024) as a marker transiently expressed as OPCs commit to differentiating, with a genuinely biphasic mechanism: early on it partners with β-catenin to inhibit differentiation (Wnt-pathway-like action), then later switches partners (HDACs, KAISO) to instead promote differentiation together with SOX10. It is separately listed as a canonical NFOL-stage marker gene in scRNA-seq marker panels (Marques et al. 2016, cited within Emery &amp; Wood 2024) — so the same transcript spans a mechanistic role at the commitment step and a marker role slightly later, at the newly-formed-oligodendrocyte stage. Not discussed in the other papers surveyed in this table. Directly confirmed: Marques et al. (2016) report that Tcf7l2 expression peaks specifically at the NFOL1/NFOL2 stage, at the same point that Gpr17 expression declines -- consistent with Emery &amp; Wood (2024)'s citation of this paper for the NFOL-marker role. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) refines the stage assignment: Tcf7l2's sharpest peak is specifically at NFOL1, with COP and NFOL2 also clearly elevated -- consistent with, and more precise than, the main text's description of a peak occurring as Gpr17 declines.</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>NFOL1 (sharpest peak; COP and NFOL2 also elevated) -- quantitative pixel analysis of Fig. S1B's single-cell heatmap; consistent with the main-text description of a peak as Gpr17 declines</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>NFOL</t>
+          <t>Newly Formed</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -2853,12 +2853,12 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>NFOL-stage marker, typically used alongside ENPP6/BCAS1 rather than alone; single-source addition here (Emery &amp; Wood 2024).</t>
+          <t>NFOL-stage marker, typically used alongside ENPP6/BCAS1 in reviews (Emery &amp; Wood 2024), and independently and extensively functionally characterized at the primary-source level by Marques et al. (2016): ITPR2+ cells are OPC-derived, newly-committed/newly-formed cells that increase with active myelination-dependent motor learning. Despite this depth of evidence, the mechanical breadth score here remains Low (only 2 of 15 paper columns) -- illustrating this table's stated limitation that Confidence reflects in-table citation breadth, not real-world marker strength.</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>Inositol 1,4,5-trisphosphate receptor type 2 (ITPR2) is grouped by Emery &amp; Wood (2024) with ENPP6 and BCAS1 as markers that together allow confident identification of newly formed oligodendrocytes, distinguishing them from more established mature cells — useful for tracking myelin repair/plasticity. Not discussed in the other papers surveyed in this table.</t>
+          <t>Inositol 1,4,5-trisphosphate receptor type 2 (ITPR2) is grouped by Emery &amp; Wood (2024) with ENPP6 and BCAS1 as markers that together allow confident identification of newly formed oligodendrocytes, distinguishing them from more established mature cells — useful for tracking myelin repair/plasticity. Not discussed in the other papers surveyed in this table. Marques et al. (2016) provide the primary functional characterization behind this marker: ITPR2+ cells are lineage-traced progeny of Pdgfra-H2B-GFP+ OPCs, are largely distinct from PDGFRA+ OPCs themselves, and show close to 100% co-positivity with SOX10 in early postnatal corpus callosum (declining with age). Critically, the number of ITPR2+/SOX10+ cells increased by ~50% after just 2 days of complex-wheel running (a motor-learning paradigm requiring active myelination) compared with non-runners -- direct evidence that this NFOL-stage marker population responds to physiological demand for new myelination, not just developmental timing. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms Itpr2's sharpest peak is at NFOL2, with COP and NFOL1 also clearly elevated -- consistent with its role marking newly-committed/newly-formed cells just after the OPC/COP transition.</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Committed precursor / Newly Formed -- sharpest peak at NFOL2 (COP and NFOL1 also elevated), quantitatively confirmed via Fig. S1B's single-cell heatmap; ~100% overlap with SOX10+ cells at these stages; %ITPR2+/SOX10+ increases ~50% after 2 days of complex-wheel motor learning vs. non-runners</t>
         </is>
       </c>
       <c r="J20" s="12" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>NFOL</t>
+          <t>Newly Formed</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -2965,12 +2965,12 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>NFOL-stage scRNA-seq marker gene; single-source, secondhand-within-a-review addition (Emery &amp; Wood 2024 citing Marques et al. 2016) — check Marques et al. 2016 directly if citing this specific marker.</t>
+          <t>NFOL-stage scRNA-seq marker gene, now directly confirmed in its primary source (Marques et al. 2016) rather than only via a secondary review's citation of it (Emery &amp; Wood 2024) -- the 'verify against the primary paper' caveat previously attached to this row is resolved.</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Listed only within the single-cell marker-gene summary in Emery &amp; Wood (2024) (itself citing Marques et al. 2016) as one of several transcripts used to define the NFOL stage; not otherwise discussed mechanistically in this review or in the other papers surveyed in this table.</t>
+          <t>Listed only within the single-cell marker-gene summary in Emery &amp; Wood (2024) (itself citing Marques et al. 2016) as one of several transcripts used to define the NFOL stage; not otherwise discussed mechanistically in this review or in the other papers surveyed in this table. Directly confirmed: Marques et al. (2016) list Casr, with Tcf7l2, as a gene induced at early stages of differentiation, specifically in NFOL1/NFOL2 cells. This is the primary source Emery &amp; Wood (2024) had cited secondhand; that citation is now independently verified.</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Newly Formed (NFOL1/NFOL2)</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>NFOL</t>
+          <t>Newly Formed</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>NFOL</t>
+          <t>Newly Formed</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>Reproducible NFOL-stage marker bridging COP and myelin-forming stages across three independent mouse sources.</t>
+          <t>Reproducible NFOL-stage marker bridging COP and myelin-forming stages across three independent mouse sources. Directly confirmed via Fig. 3A of Marques et al. (2016), where Tmem2 is shown, with Tcf7l2, Itpr2, and Pdgfa, as a gene distinguishing the COP/NFOL branch of the lineage. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a clean NFOL2 peak, cross-validating and sharpening the NFOL1/NFOL2 attribution above to specifically NFOL2.</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>NFOL1 / NFOL2</t>
+          <t>Newly Formed (NFOL1/NFOL2)</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>Most consistently cited myelination-stage marker across species. In human data (Jäkel), the OPALIN+ cluster is intermediate rather than terminal — a more distal RASGRF1+/RBFOX1+ state is generally considered the true endpoint elsewhere in the human literature, though not documented with specific marker genes in these four papers. Siletti et al. (2023) explicitly adopt the OPALIN/RBFOX1 split ‘as previously described’ by Jäkel et al. (2019), but assign the OPALIN+ population the label ‘Oligo1’ — the opposite of Jäkel's own numbering, in which RBFOX1+ (not OPALIN+) cells are ‘Oligo1’ and OPALIN+ cells form the separate cluster ‘Oligo6’. The cluster-number labels are therefore not interchangeable across these two papers even though both used the same two marker genes; only the marker-gene/biology correspondence (OPALIN = actively-myelinating/intermediate; RBFOX1 = mature/terminal) is consistent.</t>
+          <t>Most consistently cited myelination-stage marker across species. In human data (Jäkel), the OPALIN+ cluster is intermediate rather than terminal — a more distal RASGRF1+/RBFOX1+ state is generally considered the true endpoint elsewhere in the human literature, though not documented with specific marker genes in these four papers. Siletti et al. (2023) explicitly adopt the OPALIN/RBFOX1 split ‘as previously described’ by Jäkel et al. (2019), but assign the OPALIN+ population the label ‘Oligo1’ — the opposite of Jäkel's own numbering, in which RBFOX1+ (not OPALIN+) cells are ‘Oligo1’ and OPALIN+ cells form the separate cluster ‘Oligo6’. The cluster-number labels are therefore not interchangeable across these two papers even though both used the same two marker genes; only the marker-gene/biology correspondence (OPALIN = actively-myelinating/intermediate; RBFOX1 = mature/terminal) is consistent. Directly confirmed: Marques et al. (2016) group Opalin with Mal, Mog, Plp1, and Serinc5 as myelin-formation genes marking the MFOL1/MFOL2 stage -- now also independently supported by three new gene rows added to this table (MAL, MOG, SERINC5) from the same source. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a clean MFOL1 peak (MFOL2 a close second), cross-validating the MFOL1/MFOL2 attribution above.</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>MFOL1 / MFOL2</t>
+          <t>Myelinating (MFOL1/MFOL2)</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>Structural myelin gene; Jäkel et al. show it increases rather than decreases in MS mature oligodendrocytes, arguing against a simple transcriptional 'loss' of myelin genes in disease.</t>
+          <t>Structural myelin gene; Jäkel et al. show it increases rather than decreases in MS mature oligodendrocytes, arguing against a simple transcriptional 'loss' of myelin genes in disease. (Note: MAG is not one of the specific myelin-formation genes named in Marques et al. 2016's main text -- Mal, Mog, Plp1, Opalin, and Serinc5 are -- so this table's Marques2016 cell for MAG correctly remains NA despite MAG's obvious biological relevance to myelination.)</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Structural myelin gene, mature marker with early NFOL2 onset</t>
+          <t>Structural myelin gene, mature marker with early NFOL2 onset per the original secondhand citation -- this specific staging claim remains unconfirmed even after reviewing both the main text and supplementary figures S1-S16 of Marques et al. (2016); Mobp does not appear by name anywhere in either PDF. It is most likely covered only in the paper's external Table S1 ('List of 50 up-regulated genes in each branch of the dendrogram') or Table S2, which are referenced by title in the supplement but were not themselves included as data in either uploaded PDF. Treat as still-provisional pending access to those tables.</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Induced slightly earlier than PLP1/MAG in Marques et al., then maintained through terminal maturity.</t>
+          <t>Induced slightly earlier than PLP1/MAG in Marques et al., then maintained through terminal maturity. A full review of both the main text and the supplementary figures (S1-S16, including the ~139-gene single-cell heatmap in Fig. S1B) still did not locate an explicit mention of Mobp anywhere in either PDF; the NFOL2/mature-stage attribution here remains inherited from the secondhand Valihrach et al. (2022) citation. The paper's Table S1 ('List of 50 up-regulated genes in each branch of the dendrogram') and Table S2 are referenced by title on p. 24 of the supplement but are external files, not included as data in either the main-text or supplementary PDF reviewed this session -- this is the most likely source of the original claim. Verify there before citing this specific staging claim.</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>NFOL2 (early induction), sustained through mature stages</t>
+          <t>Newly Formed (early induction at NFOL2), sustained through mature stages [not found in the main text OR in the Fig. S1B single-cell heatmap gene list (~139 genes) after reviewing supplementary figures S1-S16 -- likely from an external table (e.g. Table S1/S2) not included in either PDF]</t>
         </is>
       </c>
       <c r="J27" s="12" t="inlineStr">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
-          <t>One of the highest-expressed oligodendrocyte transcripts overall in every dataset examined.</t>
+          <t>One of the highest-expressed oligodendrocyte transcripts overall in every dataset examined. Directly confirmed: Marques et al. (2016) group Plp1 with Mal, Mog, Opalin, and Serinc5 as a myelin-formation gene marking the MFOL1/MFOL2 stage in mouse.</t>
         </is>
       </c>
       <c r="H28" s="12" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="I28" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Myelinating (MFOL1/MFOL2; myelin-formation gene)</t>
         </is>
       </c>
       <c r="J28" s="12" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>Used by Mironova et al. (2026) as the standard IHC/protein marker of mature oligodendrocytes throughout their in vivo mouse imaging and immunostaining experiments (e.g., quantifying oligodendrocyte density, and showing that the great majority of transient CSPG-rich ECM structures, DACS, do not co-localize with ASPA+ cells). Emery &amp; Wood (2024) independently list aspartoacylase (ASPA) as a marker of postmitotic oligodendrocytes at the protein level (Moffett et al. 2011), consistent with Mironova's usage, and note it is typically used alongside MYRF (also now in this table) for this purpose.</t>
+          <t>Used by Mironova et al. (2026) as the standard IHC/protein marker of mature oligodendrocytes throughout their in vivo mouse imaging and immunostaining experiments (e.g., quantifying oligodendrocyte density, and showing that the great majority of transient CSPG-rich ECM structures, DACS, do not co-localize with ASPA+ cells). Emery &amp; Wood (2024) independently list aspartoacylase (ASPA) as a marker of postmitotic oligodendrocytes at the protein level (Moffett et al. 2011), consistent with Mironova's usage, and note it is typically used alongside MYRF (also now in this table) for this purpose. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms Aspa is broadly elevated across the mature MOL1-MOL6 subtypes, peaking specifically at MOL2.</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
@@ -4309,12 +4309,12 @@
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Mature-OL marker with a secondary disease/inflammation-associated signal</t>
+          <t>Mature-OL marker with a secondary disease/inflammation-associated signal. The MOL2 sub-cluster attribution for Marques2016 is now directly confirmed: quantitative pixel analysis of the single-cell heatmap in Fig. S1B shows a sharp Klk6 peak specifically at MOL2 (secondary at MOL3), matching the original citation exactly.</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
         <is>
-          <t>Unusual dual identity: a stable, healthy mature-oligodendrocyte marker (Jäkel Oligo5, Marques MOL2, Zeisel MOL3) that also recurs in inflammatory/disease gene modules (Falcão EAE, Kenigsbuch DOLs). Emery &amp; Wood (2024) independently list Klk6 (with Apod, now also in this table) as a later marker distinguishing more mature mouse oligodendrocyte populations, citing the same primary source (Marques et al. 2016) already represented as its own column in this table.</t>
+          <t>Unusual dual identity: a stable, healthy mature-oligodendrocyte marker (Jäkel Oligo5, Marques MOL2, Zeisel MOL3) that also recurs in inflammatory/disease gene modules (Falcão EAE, Kenigsbuch DOLs). Emery &amp; Wood (2024) independently list Klk6 (with Apod, now also in this table) as a later marker distinguishing more mature mouse oligodendrocyte populations, citing the same primary source (Marques et al. 2016) already represented as its own column in this table. Direct review of Marques et al. (2016)'s main text confirms Klk6 as a late/mature oligodendrocyte differentiation gene (with Apod) across MOL1-MOL6 broadly, and as the smFISH-validated 'MOL marker' (Klk6+, distinct from the MFOL marker Ctps+) in Fig. 2C. The specific 'MOL2' sub-cluster attribution, originally inherited from the secondhand Valihrach citation, is now directly confirmed: Klk6 is one of the ~139 genes plotted in the single-cell heatmap in Fig. S1B (columns ordered VLMC-&gt;OPC-&gt;COP-&gt;NFOL1-&gt;NFOL2-&gt;MFOL1-&gt;MFOL2-&gt;MOL1-&gt;MOL2-&gt;MOL3-&gt;MOL4-&gt;MOL5-&gt;MOL6), and quantitative pixel-brightness analysis of that heatmap shows Klk6's expression peaks sharply and specifically at MOL2, with a secondary peak at MOL3 and a taper through MOL4/MOL1 -- an exact match to the original citation.</t>
         </is>
       </c>
       <c r="H33" s="12" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="I33" s="12" t="inlineStr">
         <is>
-          <t>MOL2</t>
+          <t>MOL2 (peak; secondary MOL3) -- directly confirmed by quantitative pixel analysis of the single-cell heatmap in Fig. S1B</t>
         </is>
       </c>
       <c r="J33" s="12" t="inlineStr">
@@ -4421,12 +4421,12 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>Later mature-OL scRNA-seq marker gene, typically discussed alongside KLK6; single-source, secondhand-within-a-review addition (Emery &amp; Wood 2024 citing Marques et al. 2016).</t>
+          <t>Later mature-OL scRNA-seq marker gene, typically discussed alongside KLK6; now directly confirmed in its primary source (Marques et al. 2016) rather than only via secondhand citation in Emery &amp; Wood (2024).</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
-          <t>Apolipoprotein D (APOD) is listed only within the single-cell marker-gene summary in Emery &amp; Wood (2024) as one of the later markers distinguishing more mature oligodendrocyte populations, paired with KLK6 (already in this table). Not otherwise discussed mechanistically here or in the other papers surveyed in this table.</t>
+          <t>Apolipoprotein D (APOD) is listed only within the single-cell marker-gene summary in Emery &amp; Wood (2024) as one of the later markers distinguishing more mature oligodendrocyte populations, paired with KLK6 (already in this table). Not otherwise discussed mechanistically here or in the other papers surveyed in this table. Directly confirmed: Marques et al. (2016) list Apod, with Klk6, as a late oligodendrocyte differentiation gene expressed broadly across MOL1-MOL6. This is the primary source Emery &amp; Wood (2024) had cited secondhand for this marker; that citation is now independently verified. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms Apod is broadly elevated across MOL1-MOL5, peaking specifically at MOL2.</t>
         </is>
       </c>
       <c r="H34" s="12" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="I34" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Mature (MOL1-MOL6; late differentiation gene, with Klk6)</t>
         </is>
       </c>
       <c r="J34" s="12" t="inlineStr">
@@ -5200,17 +5200,17 @@
       </c>
       <c r="E41" s="18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F41" s="18" t="inlineStr">
         <is>
-          <t>Canonical pan-lineage/maturation transcription factor; continuously required for myelin gene maintenance throughout adult life, in explicit contrast to the time-limited requirement for OLIG2 (Emery &amp; Wood 2024).</t>
+          <t>Canonical pan-lineage/maturation transcription factor; continuously required for myelin gene maintenance throughout adult life (Emery &amp; Wood 2024). Now Medium by this table's own rule: broad mouse-only citation across 3 papers (Hughes2021, Emery2024, and directly-reviewed Marques et al. 2016, which uses SOX10 protein/ISH extensively as a pan-oligodendrocyte-lineage validation marker) -- though still lacking a confirmed-human citation within this table, so the true real-world consensus for this marker likely still exceeds this in-table score.</t>
         </is>
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>Master regulator of oligodendrocyte identity/myelination (SoxE family). Related SoxD-family repressors (SOX5/SOX6) oppose its action in the broader differentiation literature, though that mechanism is not detailed within these four papers. Emery &amp; Wood (2024) emphasize that, in contrast to OLIG2, continued SOX10 activity (together with MYRF, now also in this table) is necessary throughout the life of the oligodendrocyte: conditional ablation in mature cells causes severe disruption of myelin gene expression and myelin breakdown (Koenning et al. 2012).</t>
+          <t>Master regulator of oligodendrocyte identity/myelination (SoxE family). Related SoxD-family repressors (SOX5/SOX6) oppose its action in the broader differentiation literature, though that mechanism is not detailed within these four papers. Emery &amp; Wood (2024) emphasize that, in contrast to OLIG2, continued SOX10 activity (together with MYRF, now also in this table) is necessary throughout the life of the oligodendrocyte: conditional ablation in mature cells causes severe disruption of myelin gene expression and myelin breakdown (Koenning et al. 2012). Marques et al. (2016) use Sox10 extensively as a pan-oligodendrocyte-lineage marker for validation and colocalization -- e.g., smFISH confirming Sox10/Ctps/Klk6 mark distinct MFOL vs. MOL populations (Fig. 2C), and IHC quantifying %ITPR2+ among SOX10+ cells across postnatal ages (P7, P21, P90) and in the motor-learning experiment -- but Sox10 itself is not used as a differential scRNA-seq cluster marker gene in this paper (it marks essentially the whole lineage). Adding this as a third mouse-only citation (with Hughes2021 and Emery2024) raises this table's mechanical Confidence score to Medium via the 'broad mouse-only citation across &gt;=3 papers' rule -- partially, but not fully, resolving the known limitation described in the README, since this table still has no confirmed-human citation for SOX10 despite it being one of the most universally used human oligodendrocyte-lineage markers in the broader field.</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Pan-lineage (ISH/IHC pan-oligodendrocyte-lineage marker used for stage/colocalization analyses throughout -- e.g. %ITPR2+ out of SOX10+ across P7-P90 and non-runner/runner comparisons; not used as a differential scRNA-seq cluster marker in this paper)</t>
         </is>
       </c>
       <c r="J41" s="17" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="D42" s="18" t="inlineStr">
         <is>
-          <t>Immune/DAO</t>
+          <t>Immune / Disease-Associated</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="D43" s="18" t="inlineStr">
         <is>
-          <t>Immune/DAO</t>
+          <t>Immune / Disease-Associated</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="D44" s="18" t="inlineStr">
         <is>
-          <t>Immune/DAO</t>
+          <t>Immune / Disease-Associated</t>
         </is>
       </c>
       <c r="E44" s="18" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="D45" s="18" t="inlineStr">
         <is>
-          <t>Immune/DAO</t>
+          <t>Immune / Disease-Associated</t>
         </is>
       </c>
       <c r="E45" s="18" t="inlineStr">
@@ -5755,7 +5755,7 @@
       </c>
       <c r="D46" s="18" t="inlineStr">
         <is>
-          <t>Immune/DAO</t>
+          <t>Immune / Disease-Associated</t>
         </is>
       </c>
       <c r="E46" s="18" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="D47" s="18" t="inlineStr">
         <is>
-          <t>Immune/DAO</t>
+          <t>Immune / Disease-Associated</t>
         </is>
       </c>
       <c r="E47" s="18" t="inlineStr">
@@ -5877,12 +5877,12 @@
       </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
-          <t>Context-dependent: healthy terminal-subtype marker (mouse MOL6) and disease-associated signature gene (multiple pathologies)</t>
+          <t>Context-dependent: healthy terminal-subtype marker (mouse MOL6, now directly confirmed via Fig. S1B's single-cell heatmap) and disease-associated signature gene (multiple pathologies).</t>
         </is>
       </c>
       <c r="G47" s="17" t="inlineStr">
         <is>
-          <t>A gene that is a baseline marker of a normal mature mouse subtype (MOL6) in Marques et al. but becomes part of the disease-associated signature in later studies — the same transcript can mark a healthy terminal state and a reactive state, so it should not be used as a disease marker in isolation from cluster context.</t>
+          <t>A gene that is a baseline marker of a normal mature mouse subtype (MOL6) in Marques et al. but becomes part of the disease-associated signature in later studies — the same transcript can mark a healthy terminal state and a reactive state, so it should not be used as a disease marker in isolation from cluster context. Il33 is not named in the main text, but it is one of the ~139 genes plotted in the single-cell heatmap in Fig. S1B of the supplementary materials. Quantitative pixel-brightness analysis of that heatmap shows a sharp, isolated Il33 peak specifically at MOL6 (next-highest cluster, MOL5, is far lower) -- directly confirming the MOL6/homeostatic attribution inherited from the secondhand Valihrach et al. (2022) citation.</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>MOL6 (healthy, homeostatic mature subtype)</t>
+          <t>MOL6 (healthy, homeostatic mature subtype) -- directly confirmed by quantitative pixel analysis of the single-cell heatmap in Fig. S1B (sharp, isolated MOL6 peak)</t>
         </is>
       </c>
       <c r="J47" s="17" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="D48" s="18" t="inlineStr">
         <is>
-          <t>MHC/Interferon</t>
+          <t>Histocompatibility / Interferon</t>
         </is>
       </c>
       <c r="E48" s="18" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="D49" s="18" t="inlineStr">
         <is>
-          <t>MHC/Interferon</t>
+          <t>Histocompatibility / Interferon</t>
         </is>
       </c>
       <c r="E49" s="18" t="inlineStr">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="D50" s="18" t="inlineStr">
         <is>
-          <t>MHC/Interferon</t>
+          <t>Histocompatibility / Interferon</t>
         </is>
       </c>
       <c r="E50" s="18" t="inlineStr">
@@ -6969,8 +6969,1016 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>NEU4</t>
+        </is>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>COP / early differentiating</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Committed Precursor</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>Mouse COP-stage marker gene; single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G57" s="12" t="inlineStr">
+        <is>
+          <t>Sialidase family gene (neuraminidase 4) expressed by differentiation-committed oligodendrocyte precursors (COPs) once they lose Pdgfra/Cspg4 expression, per Marques et al. (2016). Not discussed in the other papers surveyed in this table; function in COPs not elaborated beyond marker use. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms a clean COP peak, cross-validating the COP attribution above.</t>
+        </is>
+      </c>
+      <c r="H57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I57" s="12" t="inlineStr">
+        <is>
+          <t>Committed Precursor (COP)</t>
+        </is>
+      </c>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q57" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R57" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S57" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T57" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U57" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V57" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>MAL</t>
+        </is>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>Myelinating (structural)</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Myelinating</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>Mouse myelin-formation structural gene; single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>Myelin and lymphocyte protein (MAL) is one of five genes Marques et al. (2016) group together as responsible for myelin formation in MFOL1/MFOL2 (with Mog, Plp1, Opalin, Serinc5). Not discussed in the other papers surveyed in this table.</t>
+        </is>
+      </c>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>MFOL1 / MFOL2</t>
+        </is>
+      </c>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q58" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R58" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S58" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T58" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U58" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V58" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="90" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>MOG</t>
+        </is>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>Myelinating (structural)</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>Myelinating</t>
+        </is>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>Mouse myelin-formation structural gene; single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G59" s="12" t="inlineStr">
+        <is>
+          <t>Myelin oligodendrocyte glycoprotein (MOG), grouped by Marques et al. (2016) with Mal, Plp1, Opalin, and Serinc5 as myelin-formation genes in MFOL1/MFOL2. Widely used elsewhere in the field as a myelin-sheath surface marker, but not independently discussed in the other papers surveyed in this table.</t>
+        </is>
+      </c>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I59" s="12" t="inlineStr">
+        <is>
+          <t>MFOL1 / MFOL2</t>
+        </is>
+      </c>
+      <c r="J59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q59" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R59" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S59" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T59" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U59" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V59" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="90" customHeight="1">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>SERINC5</t>
+        </is>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>Myelinating</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Myelinating</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>Mouse myelin-formation gene; single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G60" s="12" t="inlineStr">
+        <is>
+          <t>Serine incorporator 5, grouped by Marques et al. (2016) with Mal, Mog, Plp1, and Opalin as myelin-formation genes in MFOL1/MFOL2. Not discussed in the other papers surveyed in this table.</t>
+        </is>
+      </c>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>MFOL1 / MFOL2</t>
+        </is>
+      </c>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q60" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R60" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S60" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T60" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U60" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V60" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="90" customHeight="1">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>TRF</t>
+        </is>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>Myelinating (iron transport; transferrin)</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>Myelinating</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>Mouse myelinating-stage gene (transferrin); single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>Transferrin, listed by Marques et al. (2016) as one of two genes "present in myelinating cells" (with Pmp22) in mature oligodendrocytes (MOL1-MOL6). Transferrin is also produced by other CNS cell types (e.g., choroid plexus epithelium), so use with caution as a standalone oligodendrocyte marker. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms Trf is broadly elevated across MOL1-MOL5, peaking specifically at MOL2.</t>
+        </is>
+      </c>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="inlineStr">
+        <is>
+          <t>MOL1-MOL6 (myelinating cells)</t>
+        </is>
+      </c>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q61" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R61" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S61" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T61" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U61" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V61" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="90" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>PMP22</t>
+        </is>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>Myelinating (structural; also differentiates MOL1-4 lipid-biosynthesis/myelination genes from MOL5/MOL6)</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Myelinating</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>Mouse myelinating/mature-stage structural gene; single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>Peripheral myelin protein 22, listed by Marques et al. (2016) as present in myelinating cells (with Trf) across MOL1-MOL6, and separately as one of the lipid-biosynthesis/myelination genes (with Far1) that differentiate MOL1-MOL4 from the more synapse-associated MOL5/MOL6 subtypes. Better known as a peripheral (Schwann cell) myelin gene; its central-oligodendrocyte role is comparatively less established outside this paper. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) confirms Pmp22 is broadly elevated across MOL1-MOL5, peaking specifically at MOL2.</t>
+        </is>
+      </c>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I62" s="12" t="inlineStr">
+        <is>
+          <t>MOL1-MOL4 (with Far1); also broadly MOL1-MOL6 (myelinating cells, with Trf)</t>
+        </is>
+      </c>
+      <c r="J62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q62" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R62" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S62" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T62" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U62" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V62" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="90" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>FAR1</t>
+        </is>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>Mature (lipid biosynthesis; differentiates MOL1-4 from MOL5/MOL6)</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>Mouse mature-oligodendrocyte subtype gene (lipid biosynthesis); single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>Fatty acyl-CoA reductase 1, identified by gene ontology analysis as enriched in MOL1-MOL4 (lipid biosynthesis and myelination genes, with Pmp22), distinguishing this subset from the more synapse-associated adult subtypes MOL5/MOL6. Not discussed in the other papers surveyed in this table.</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I63" s="12" t="inlineStr">
+        <is>
+          <t>MOL1-MOL4</t>
+        </is>
+      </c>
+      <c r="J63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q63" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R63" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S63" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T63" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U63" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V63" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="90" customHeight="1">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>GRM3</t>
+        </is>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>Mature (synapse-associated; broadly elevated across mature MOL1-MOL6 subtypes, not MOL6-specific)</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>Mouse mature-oligodendrocyte gene (metabotropic glutamate receptor), broadly elevated across the mature MOL1-MOL6 subtypes rather than sharply restricted to one; single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G64" s="12" t="inlineStr">
+        <is>
+          <t>Metabotropic glutamate receptor 3, discussed by Marques et al. (2016) as a gene marking synapse-associated signaling in mature oligodendrocytes, confirmed at the protein level in Pdgfra-Cre-RCE traced, CC1+ mature oligodendrocytes in the juvenile cortex. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) shows Grm3 broadly elevated across MOL1 through MOL6, with only a mild, non-specific lean toward MOL4/MOL5/MOL6 -- correcting an earlier draft note in this table that had (incorrectly) described it as 'MOL6 mainly' before this heatmap was available. Illustrates that some mature oligodendrocyte subtypes carry synaptic-signaling machinery rather than purely myelination genes. Not discussed in the other papers surveyed in this table.</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I64" s="12" t="inlineStr">
+        <is>
+          <t>Broadly elevated across MOL1-MOL6 (nominal peak at MOL5, close to MOL4/MOL6) -- quantitative pixel analysis of Fig. S1B's single-cell heatmap; correction of an earlier 'MOL6 mainly' draft assignment made before this heatmap was reviewed</t>
+        </is>
+      </c>
+      <c r="J64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q64" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R64" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S64" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T64" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U64" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V64" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="90" customHeight="1">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>JPH4</t>
+        </is>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>Maturation identity</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>Mature (synapse-associated; MOL5-peaking, MOL6 close second, alongside GRM3)</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>Mouse mature-oligodendrocyte subtype gene (junctophilin, synapse-associated); single-source addition (Marques et al. 2016).</t>
+        </is>
+      </c>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>Junctophilin 4, identified alongside GRM3 as a synapse-related gene enriched in mature adult oligodendrocyte subtypes. Quantitative pixel analysis of the single-cell heatmap in Fig. S1B (supplementary materials) shows Jph4's peak is specifically at MOL5, with MOL6 a close second -- correcting an earlier draft note in this table that had described it simply as 'MOL6' before this heatmap was available. Not discussed in the other papers surveyed in this table.</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I65" s="12" t="inlineStr">
+        <is>
+          <t>MOL5 (peak; MOL6 a close second) -- quantitative pixel analysis of Fig. S1B's single-cell heatmap; correction of an earlier 'MOL6' draft assignment made before this heatmap was reviewed</t>
+        </is>
+      </c>
+      <c r="J65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q65" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R65" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S65" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T65" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U65" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V65" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V56"/>
+  <autoFilter ref="A1:V65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -7180,7 +8188,7 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Not directly reviewed this session; marker genes taken from Valihrach et al. 2022 Table 2. Verify against the primary paper before citing.</t>
+          <t>Uploaded PDF (main text + figures) AND supplementary materials (Figs. S1-S16, incl. the ~139-gene single-cell heatmap in Fig. S1B); both reviewed directly this session. The KLK6 MOL2 sub-cluster claim and the IL33 MOL6 claim -- both originally inherited from the secondhand Valihrach citation -- are now directly confirmed via quantitative pixel-brightness analysis of the Fig. S1B single-cell heatmap (Klk6 peaks sharply at MOL2; Il33 peaks sharply and specifically at MOL6). The MOBP NFOL2-onset stage claim remains unresolved: Mobp does not appear by name in either the main text or the supplementary figures; it most likely traces to the paper's external Table S1 ('List of 50 up-regulated genes in each branch of the dendrogram') or Table S2, which are referenced by title on p. 24 of the supplement but were not included as data in either PDF reviewed this session. All other Marques2016 attributions in this table (OPC, COP, NFOL, MFOL, and MOL1-MOL6 marker genes; VLMC caveat; ITPR2 motor-learning functional data; SOX10 pan-lineage validation use) were confirmed directly from the main text and figures, several further cross-validated quantitatively against Fig. S1B.</t>
         </is>
       </c>
     </row>

</xml_diff>